<commit_message>
refactor: change gojs to mermaid, add multilingual, update crf_* structure model
</commit_message>
<xml_diff>
--- a/src/staticfiles/study/templates/crf_templates_import_template.xlsx
+++ b/src/staticfiles/study/templates/crf_templates_import_template.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="CRF Templates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Page Templates" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,25 +26,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001E2B36"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAF7"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,20 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="009FB9D1"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,28 +414,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Vi Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>En Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>Version</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CRF Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Vi Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>En Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Order</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix logic form template
</commit_message>
<xml_diff>
--- a/src/staticfiles/study/templates/crf_templates_import_template.xlsx
+++ b/src/staticfiles/study/templates/crf_templates_import_template.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CRF Templates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Form Templates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Section Templates" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,4 +442,65 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Form Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Vi Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>En Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Repeated</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Min Repeat</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Max Repeat</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>